<commit_message>
auto: sensor data update
</commit_message>
<xml_diff>
--- a/solar_log.xlsx
+++ b/solar_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,6 +538,21 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-17 17:50:03</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>35</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>OK(FC03)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>